<commit_message>
Output quality round: charts, formula rows, deduplicated findings
The deck summary slide now carries real data visualization: a revenue
column chart and a separate EBITDA margin line chart, single series
each, directly labeled, no gridlines. The business summary findings
box compresses to one liners instead of repeating Section 2, and the
financial table gains a revenue growth percent row. The Excel
workbook gains live growth and margin formula rows in Historicals and
a total as percent of revenue row in the model.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/financial_Model.xlsx
+++ b/samples/financial_Model.xlsx
@@ -523,7 +523,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <cols>
     <col min="1" max="1" width="42.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -615,21 +615,38 @@
         <v>21.0641</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="str">
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Total as % of target revenue</v>
+      </c>
+      <c r="B7" s="2">
+        <f>B6/Inputs!$B$4</f>
+        <v>0.05921338797814208</v>
+      </c>
+      <c r="C7" s="2">
+        <f>C6/Inputs!$B$4</f>
+        <v>0.08715887978142077</v>
+      </c>
+      <c r="D7" s="2">
+        <f>D6/Inputs!$B$4</f>
+        <v>0.11510437158469945</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
         <v>All cells on this sheet are formulas driven by the Inputs sheet.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -723,9 +740,47 @@
         <v>34.3</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Revenue growth (%)</v>
+      </c>
+      <c r="C6" s="2">
+        <f>(C2-B2)/B2</f>
+        <v>0.08450704225352124</v>
+      </c>
+      <c r="D6" s="2">
+        <f>(D2-C2)/C2</f>
+        <v>0.09090909090909083</v>
+      </c>
+      <c r="E6" s="2">
+        <f>(E2-D2)/D2</f>
+        <v>0.08928571428571419</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>EBITDA margin (%)</v>
+      </c>
+      <c r="B7" s="2">
+        <f>B5/B2</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="C7" s="2">
+        <f>C5/C2</f>
+        <v>0.16103896103896106</v>
+      </c>
+      <c r="D7" s="2">
+        <f>D5/D2</f>
+        <v>0.17261904761904762</v>
+      </c>
+      <c r="E7" s="2">
+        <f>E5/E2</f>
+        <v>0.18743169398907103</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sensitivity grid, Method page, sample downloads, GitHub link
The Valuation sheet gains a five by five enterprise value sensitivity
grid across growth and multiple, all live formulas around the input
base case, labeled on next year EBITDA to avoid a mixed basis with
the point estimate. A plain language Method page explains the engine
task by task on the PwC structure, including what it cannot do. The
deliverables band links directly to finished sample files, and the
footer links to the source.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/financial_Model.xlsx
+++ b/samples/financial_Model.xlsx
@@ -35,7 +35,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
-  <numFmts count="8">
+  <numFmts count="10">
     <numFmt numFmtId="165" formatCode="#,##0.0;(#,##0.0)"/>
     <numFmt numFmtId="166" formatCode="#,##0.0;(#,##0.0)"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
@@ -44,8 +44,10 @@
     <numFmt numFmtId="170" formatCode="#,##0.0;(#,##0.0)"/>
     <numFmt numFmtId="171" formatCode="#,##0.0;(#,##0.0)"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
+    <numFmt numFmtId="173" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="174" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -166,8 +168,20 @@
       <b/>
       <color rgb="1A1A1A"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+      <color rgb="FFFFFF"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <b/>
+      <color rgb="0A1F2E"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="18">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -259,6 +273,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F5F7"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0A1F2E"/>
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8EDFF"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -378,7 +404,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -425,6 +451,12 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="173" fontId="21" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="22" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1346,7 +1378,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:F23"/>
   <cols>
     <col min="1" max="1" width="46.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1450,9 +1482,189 @@
         <v>274.5</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="6" t="str">
+        <v>SENSITIVITY: EV ON NEXT YEAR EBITDA, ACROSS GROWTH AND MULTIPLE</v>
+      </c>
+      <c r="B16" s="6" t="str">
+        <v/>
+      </c>
+      <c r="C16" s="6" t="str">
+        <v/>
+      </c>
+      <c r="D16" s="6" t="str">
+        <v/>
+      </c>
+      <c r="E16" s="6" t="str">
+        <v/>
+      </c>
+      <c r="F16" s="6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="str">
+        <v>Growth below, multiple right</v>
+      </c>
+      <c r="B17" s="22">
+        <f>Inputs!$B$23+-2</f>
+        <v>6</v>
+      </c>
+      <c r="C17" s="22">
+        <f>Inputs!$B$23+-1</f>
+        <v>7</v>
+      </c>
+      <c r="D17" s="22">
+        <f>Inputs!$B$23+0</f>
+        <v>8</v>
+      </c>
+      <c r="E17" s="22">
+        <f>Inputs!$B$23+1</f>
+        <v>9</v>
+      </c>
+      <c r="F17" s="22">
+        <f>Inputs!$B$23+2</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23">
+        <f>Inputs!$B$10+-0.02</f>
+        <v>0.06823055346886432</v>
+      </c>
+      <c r="B18" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <v>219.8418479038923</v>
+      </c>
+      <c r="C18" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <v>256.48215588787434</v>
+      </c>
+      <c r="D18" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <v>293.1224638718564</v>
+      </c>
+      <c r="E18" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <v>329.7627718558384</v>
+      </c>
+      <c r="F18" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <v>366.40307983982046</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23">
+        <f>Inputs!$B$10+-0.01</f>
+        <v>0.07823055346886433</v>
+      </c>
+      <c r="B19" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <v>221.89984790389227</v>
+      </c>
+      <c r="C19" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <v>258.8831558878743</v>
+      </c>
+      <c r="D19" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <v>295.86646387185635</v>
+      </c>
+      <c r="E19" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <v>332.8497718558384</v>
+      </c>
+      <c r="F19" s="16">
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <v>369.83307983982047</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23">
+        <f>Inputs!$B$10+0</f>
+        <v>0.08823055346886433</v>
+      </c>
+      <c r="B20" s="16">
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <v>223.9578479038923</v>
+      </c>
+      <c r="C20" s="16">
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <v>261.28415588787436</v>
+      </c>
+      <c r="D20" s="19">
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <v>298.6104638718564</v>
+      </c>
+      <c r="E20" s="16">
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <v>335.9367718558384</v>
+      </c>
+      <c r="F20" s="16">
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <v>373.2630798398205</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23">
+        <f>Inputs!$B$10+0.01</f>
+        <v>0.09823055346886432</v>
+      </c>
+      <c r="B21" s="16">
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <v>226.01584790389228</v>
+      </c>
+      <c r="C21" s="16">
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <v>263.6851558878743</v>
+      </c>
+      <c r="D21" s="16">
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <v>301.35446387185635</v>
+      </c>
+      <c r="E21" s="16">
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <v>339.0237718558384</v>
+      </c>
+      <c r="F21" s="16">
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <v>376.6930798398204</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23">
+        <f>Inputs!$B$10+0.02</f>
+        <v>0.10823055346886433</v>
+      </c>
+      <c r="B22" s="16">
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <v>228.07384790389224</v>
+      </c>
+      <c r="C22" s="16">
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <v>266.08615588787427</v>
+      </c>
+      <c r="D22" s="16">
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <v>304.0984638718563</v>
+      </c>
+      <c r="E22" s="16">
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <v>342.1107718558384</v>
+      </c>
+      <c r="F22" s="16">
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <v>380.12307983982043</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="str">
+        <v>EBITDA in each cell is next year revenue at that growth times the current margin.</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix slides rendering on a 10 inch canvas and Word pages as A4
The deck laid every element out on a 13.333 by 7.5 inch grid but
declared LAYOUT_16x9, which pptxgenjs defines as 10 by 5.625 inches.
The right quarter of every slide and everything below 5.6 inches,
including the takeaway bar, source line, and page number, therefore
hung off the page. The canvas is now declared explicitly. Word
documents were inheriting the library default of A4 and are now
US Letter.

Both defects came from trusting a library default and from checkers
that hardcoded the same assumption as the generator. The geometry
checker now reads the slide size out of presentation.xml, and the
adversarial suite asserts both the slide canvas and the page size.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/financial_Model.xlsx
+++ b/samples/financial_Model.xlsx
@@ -788,7 +788,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B23"/>
   <cols>
     <col min="1" max="1" width="48.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -852,105 +852,97 @@
         <v>0.08823055346886433</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="str">
-        <v>EBITDA margin, projection years</v>
-      </c>
-      <c r="B11" s="10">
-        <v>0.187</v>
+    <row r="12">
+      <c r="A12" s="6" t="str">
+        <v>SYNERGY ASSUMPTIONS, EACH APPLIED TO ITS OWN LINE</v>
+      </c>
+      <c r="B12" s="6" t="str">
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="str">
-        <v>SYNERGY ASSUMPTIONS, EACH APPLIED TO ITS OWN LINE</v>
-      </c>
-      <c r="B13" s="6" t="str">
-        <v/>
+      <c r="A13" s="7" t="str">
+        <v>Revenue uplift, low end</v>
+      </c>
+      <c r="B13" s="10">
+        <v>0.05</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="str">
-        <v>Revenue uplift, low end</v>
+        <v>Revenue uplift, high end</v>
       </c>
       <c r="B14" s="10">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="str">
-        <v>Revenue uplift, high end</v>
+        <v>Flow through margin on new revenue</v>
       </c>
       <c r="B15" s="10">
-        <v>0.1</v>
+        <v>0.187</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="str">
-        <v>Flow through margin on new revenue</v>
+        <v>Cost of goods sold: synergy %, low end</v>
       </c>
       <c r="B16" s="10">
-        <v>0.187</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="str">
-        <v>Cost of goods sold: synergy %, low end</v>
+        <v>Cost of goods sold: synergy %, high end</v>
       </c>
       <c r="B17" s="10">
-        <v>0.05</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="str">
-        <v>Cost of goods sold: synergy %, high end</v>
+        <v>Opex / G&amp;A (back office): synergy %, low end</v>
       </c>
       <c r="B18" s="10">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="str">
-        <v>Opex / G&amp;A (back office): synergy %, low end</v>
+        <v>Opex / G&amp;A (back office): synergy %, high end</v>
       </c>
       <c r="B19" s="10">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="7" t="str">
-        <v>Opex / G&amp;A (back office): synergy %, high end</v>
-      </c>
-      <c r="B20" s="10">
         <v>0.25</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="6" t="str">
+        <v>VALUATION ASSUMPTIONS</v>
+      </c>
+      <c r="B21" s="6" t="str">
+        <v/>
+      </c>
+    </row>
     <row r="22">
-      <c r="A22" s="6" t="str">
-        <v>VALUATION ASSUMPTIONS</v>
-      </c>
-      <c r="B22" s="6" t="str">
-        <v/>
+      <c r="A22" s="7" t="str">
+        <v>EV to EBITDA multiple</v>
+      </c>
+      <c r="B22" s="11">
+        <v>8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="str">
-        <v>EV to EBITDA multiple</v>
+        <v>EV to revenue multiple, cross check</v>
       </c>
       <c r="B23" s="11">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="str">
-        <v>EV to revenue multiple, cross check</v>
-      </c>
-      <c r="B24" s="11">
         <v>1.5</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1289,15 +1281,15 @@
         <v>Revenue synergy, at flow through margin</v>
       </c>
       <c r="B4" s="16">
-        <f>Inputs!$B$5*Inputs!$B$14*Inputs!$B$16</f>
+        <f>Inputs!$B$5*Inputs!$B$13*Inputs!$B$15</f>
         <v>1.71105</v>
       </c>
       <c r="C4" s="16">
-        <f>Inputs!$B$5*AVERAGE(Inputs!$B$14,Inputs!$B$15)*Inputs!$B$16</f>
+        <f>Inputs!$B$5*AVERAGE(Inputs!$B$13,Inputs!$B$14)*Inputs!$B$15</f>
         <v>2.5665750000000003</v>
       </c>
       <c r="D4" s="16">
-        <f>Inputs!$B$5*Inputs!$B$15*Inputs!$B$16</f>
+        <f>Inputs!$B$5*Inputs!$B$14*Inputs!$B$15</f>
         <v>3.4221</v>
       </c>
     </row>
@@ -1306,15 +1298,15 @@
         <v>Cost of goods sold synergy</v>
       </c>
       <c r="B5" s="16">
+        <f>Inputs!$B$6*Inputs!$B$16</f>
+        <v>5.745000000000001</v>
+      </c>
+      <c r="C5" s="16">
+        <f>Inputs!$B$6*AVERAGE(Inputs!$B$16,Inputs!$B$17)</f>
+        <v>7.468500000000001</v>
+      </c>
+      <c r="D5" s="16">
         <f>Inputs!$B$6*Inputs!$B$17</f>
-        <v>5.745000000000001</v>
-      </c>
-      <c r="C5" s="16">
-        <f>Inputs!$B$6*AVERAGE(Inputs!$B$17,Inputs!$B$18)</f>
-        <v>7.468500000000001</v>
-      </c>
-      <c r="D5" s="16">
-        <f>Inputs!$B$6*Inputs!$B$18</f>
         <v>9.192</v>
       </c>
     </row>
@@ -1323,15 +1315,15 @@
         <v>Opex / G&amp;A (back office) synergy</v>
       </c>
       <c r="B6" s="16">
+        <f>Inputs!$B$7*Inputs!$B$18</f>
+        <v>3.38</v>
+      </c>
+      <c r="C6" s="16">
+        <f>Inputs!$B$7*AVERAGE(Inputs!$B$18,Inputs!$B$19)</f>
+        <v>5.914999999999999</v>
+      </c>
+      <c r="D6" s="16">
         <f>Inputs!$B$7*Inputs!$B$19</f>
-        <v>3.38</v>
-      </c>
-      <c r="C6" s="16">
-        <f>Inputs!$B$7*AVERAGE(Inputs!$B$19,Inputs!$B$20)</f>
-        <v>5.914999999999999</v>
-      </c>
-      <c r="D6" s="16">
-        <f>Inputs!$B$7*Inputs!$B$20</f>
         <v>8.45</v>
       </c>
     </row>
@@ -1416,7 +1408,7 @@
         <v>Enterprise value at the multiple</v>
       </c>
       <c r="B6" s="16">
-        <f>B5*Inputs!$B$23</f>
+        <f>B5*Inputs!$B$22</f>
         <v>274.4</v>
       </c>
     </row>
@@ -1443,7 +1435,7 @@
         <v>Enterprise value including synergy capture</v>
       </c>
       <c r="B9" s="16">
-        <f>B8*Inputs!$B$23</f>
+        <f>B8*Inputs!$B$22</f>
         <v>402.00059999999996</v>
       </c>
     </row>
@@ -1478,7 +1470,7 @@
         <v>Enterprise value at the revenue multiple</v>
       </c>
       <c r="B14" s="16">
-        <f>B13*Inputs!$B$24</f>
+        <f>B13*Inputs!$B$23</f>
         <v>274.5</v>
       </c>
     </row>
@@ -1507,23 +1499,23 @@
         <v>Growth below, multiple right</v>
       </c>
       <c r="B17" s="22">
-        <f>Inputs!$B$23+-2</f>
+        <f>Inputs!$B$22+-2</f>
         <v>6</v>
       </c>
       <c r="C17" s="22">
-        <f>Inputs!$B$23+-1</f>
+        <f>Inputs!$B$22+-1</f>
         <v>7</v>
       </c>
       <c r="D17" s="22">
-        <f>Inputs!$B$23+0</f>
+        <f>Inputs!$B$22+0</f>
         <v>8</v>
       </c>
       <c r="E17" s="22">
-        <f>Inputs!$B$23+1</f>
+        <f>Inputs!$B$22+1</f>
         <v>9</v>
       </c>
       <c r="F17" s="22">
-        <f>Inputs!$B$23+2</f>
+        <f>Inputs!$B$22+2</f>
         <v>10</v>
       </c>
     </row>
@@ -1533,23 +1525,23 @@
         <v>0.06823055346886432</v>
       </c>
       <c r="B18" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$22+-2)</f>
         <v>219.8418479038923</v>
       </c>
       <c r="C18" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$22+-1)</f>
         <v>256.48215588787434</v>
       </c>
       <c r="D18" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$22+0)</f>
         <v>293.1224638718564</v>
       </c>
       <c r="E18" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$22+1)</f>
         <v>329.7627718558384</v>
       </c>
       <c r="F18" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <f>B13*(1+Inputs!$B$10+-0.02)*(B5/B13)*(Inputs!$B$22+2)</f>
         <v>366.40307983982046</v>
       </c>
     </row>
@@ -1559,23 +1551,23 @@
         <v>0.07823055346886433</v>
       </c>
       <c r="B19" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$22+-2)</f>
         <v>221.89984790389227</v>
       </c>
       <c r="C19" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$22+-1)</f>
         <v>258.8831558878743</v>
       </c>
       <c r="D19" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$22+0)</f>
         <v>295.86646387185635</v>
       </c>
       <c r="E19" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$22+1)</f>
         <v>332.8497718558384</v>
       </c>
       <c r="F19" s="16">
-        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <f>B13*(1+Inputs!$B$10+-0.01)*(B5/B13)*(Inputs!$B$22+2)</f>
         <v>369.83307983982047</v>
       </c>
     </row>
@@ -1585,23 +1577,23 @@
         <v>0.08823055346886433</v>
       </c>
       <c r="B20" s="16">
-        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$22+-2)</f>
         <v>223.9578479038923</v>
       </c>
       <c r="C20" s="16">
-        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$22+-1)</f>
         <v>261.28415588787436</v>
       </c>
       <c r="D20" s="19">
-        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$22+0)</f>
         <v>298.6104638718564</v>
       </c>
       <c r="E20" s="16">
-        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$22+1)</f>
         <v>335.9367718558384</v>
       </c>
       <c r="F20" s="16">
-        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <f>B13*(1+Inputs!$B$10+0)*(B5/B13)*(Inputs!$B$22+2)</f>
         <v>373.2630798398205</v>
       </c>
     </row>
@@ -1611,23 +1603,23 @@
         <v>0.09823055346886432</v>
       </c>
       <c r="B21" s="16">
-        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$22+-2)</f>
         <v>226.01584790389228</v>
       </c>
       <c r="C21" s="16">
-        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$22+-1)</f>
         <v>263.6851558878743</v>
       </c>
       <c r="D21" s="16">
-        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$22+0)</f>
         <v>301.35446387185635</v>
       </c>
       <c r="E21" s="16">
-        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$22+1)</f>
         <v>339.0237718558384</v>
       </c>
       <c r="F21" s="16">
-        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <f>B13*(1+Inputs!$B$10+0.01)*(B5/B13)*(Inputs!$B$22+2)</f>
         <v>376.6930798398204</v>
       </c>
     </row>
@@ -1637,23 +1629,23 @@
         <v>0.10823055346886433</v>
       </c>
       <c r="B22" s="16">
-        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+-2)</f>
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$22+-2)</f>
         <v>228.07384790389224</v>
       </c>
       <c r="C22" s="16">
-        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+-1)</f>
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$22+-1)</f>
         <v>266.08615588787427</v>
       </c>
       <c r="D22" s="16">
-        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+0)</f>
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$22+0)</f>
         <v>304.0984638718563</v>
       </c>
       <c r="E22" s="16">
-        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+1)</f>
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$22+1)</f>
         <v>342.1107718558384</v>
       </c>
       <c r="F22" s="16">
-        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$23+2)</f>
+        <f>B13*(1+Inputs!$B$10+0.02)*(B5/B13)*(Inputs!$B$22+2)</f>
         <v>380.12307983982043</v>
       </c>
     </row>

</xml_diff>